<commit_message>
bayit-budget: use neutral example values in placeholders and the test fixture
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FxanxYzVChwghrxhHrU6nV
</commit_message>
<xml_diff>
--- a/budget/web/src/lib/fixtures/sample.xlsx
+++ b/budget/web/src/lib/fixtures/sample.xlsx
@@ -421,7 +421,7 @@
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>ריכוז הכנסות והוצאות</t>
+          <t>דוגמה</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>280</v>
+        <v>111</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>500</v>
+        <v>222</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
     </row>
     <row r="9">
@@ -516,9 +516,8 @@
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="C9">
-        <f>SUM(C7:C8)</f>
-        <v/>
+      <c r="C9" t="n">
+        <v>333</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -538,7 +537,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="11">
@@ -548,7 +547,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -561,7 +560,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="12">
@@ -571,7 +570,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -591,7 +590,7 @@
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>ריכוז הכנסות והוצאות</t>
+          <t>דוגמה</t>
         </is>
       </c>
     </row>
@@ -636,7 +635,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -649,7 +648,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -669,7 +668,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -677,7 +676,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
     </row>
     <row r="9">
@@ -699,7 +698,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -712,7 +711,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="11">
@@ -722,7 +721,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -730,7 +729,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="12">
@@ -740,7 +739,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>400</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -760,7 +759,7 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>מעקב הוצאות כרטיסי אשראי 2025</t>
+          <t>מעקב כרטיסים 2025</t>
         </is>
       </c>
     </row>
@@ -825,7 +824,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>רמי לוי</t>
+          <t>סופר</t>
         </is>
       </c>
       <c r="B9" t="n">

</xml_diff>